<commit_message>
Publish Auronzo_2023_JWCH, Barnaul_2021_WC, Belgrade_2017_WC, Copenhagen_2021_WCH, Duisburg_2015_WC, Duisburg_2016_WC, Duisburg_2019_WC, Duisburg_2023_WCH, Halifax_2022_WCH, Montemor_2017_WC, Montemor_2018_WCH, Montemor_2021_JWCH, Montemor_2025_JWCH, Paris_2024_OG, Pitesti_2017_JWCH, Pitesti_2019_JWCH, Plovdiv_2018_JWCH, Plovdiv_2024_JWCH, Poznan_2019_WC, Poznan_2022_WC, Poznan_2024_WC, Poznan_2025_WC, Racice_2017_WCH, Racice_2022_WC, Samarkand_2024_WCH, Szeged_2019_WCH, Szeged_2021_WC, Szeged_2022_JWCH, Szeged_2024_WC, Szeged_2025_WC, Tokyo_2021_OG, Welland_2013_JWCH
</commit_message>
<xml_diff>
--- a/events/Barnaul_2021_WC/Barnaul_2021_WC_Results.xlsx
+++ b/events/Barnaul_2021_WC/Barnaul_2021_WC_Results.xlsx
@@ -17431,6 +17431,11 @@
           <t>00:00:47.536</t>
         </is>
       </c>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>95617</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -28277,6 +28282,11 @@
           <t>00:00:47.155</t>
         </is>
       </c>
+      <c r="R429" t="inlineStr">
+        <is>
+          <t>95617</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -34132,6 +34142,11 @@
           <t>00:00:48.736</t>
         </is>
       </c>
+      <c r="R519" t="inlineStr">
+        <is>
+          <t>95617</t>
+        </is>
+      </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -40628,6 +40643,11 @@
           <t>00:02:02.371</t>
         </is>
       </c>
+      <c r="R618" t="inlineStr">
+        <is>
+          <t>95617</t>
+        </is>
+      </c>
       <c r="S618" t="inlineStr">
         <is>
           <t>100406</t>
@@ -44659,6 +44679,11 @@
       <c r="P677" t="inlineStr">
         <is>
           <t>00:26:54.438</t>
+        </is>
+      </c>
+      <c r="R677" t="inlineStr">
+        <is>
+          <t>95617</t>
         </is>
       </c>
     </row>
@@ -46319,7 +46344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D166"/>
+  <dimension ref="A1:D167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49974,6 +49999,28 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>95617</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Yarisleidis</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>CIRILO DUBOYS</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish Brandenburg_2026_WC, Poznan_2026_WC, Poznan_2025_WC, Gyor_2025_MAR, Szeged_2024_WC, Samarkand_2024_WCH, Poznan_2024_WC, Plovdiv_2024_JWCH, Paris_2024_PG, Paris_2024_OG, Metkovic_2024_MAR, Vejen_2023_MAR, Szeged_2023_WC, Poznan_2023_WC, Duisburg_2023_WCH, Auronzo_2023_JWCH, Szeged_2022_JWCH, Racice_2022_WC, Poznan_2022_WC, PonteDeLima_2022_MAR, Halifax_2022_WCH, Birmingham_2022_TWG, Tokyo_2021_OG, Szeged_2021_WC, Pitesti_2021_MAR, Moscow_2021_MAR, Montemor_2021_JWCH, Copenhagen_2021_WCH, Barnaul_2021_WC
</commit_message>
<xml_diff>
--- a/events/Barnaul_2021_WC/Barnaul_2021_WC_Results.xlsx
+++ b/events/Barnaul_2021_WC/Barnaul_2021_WC_Results.xlsx
@@ -1890,6 +1890,11 @@
           <t>00:00:43.224</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>36164</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3173,6 +3178,11 @@
           <t>00:00:44.453</t>
         </is>
       </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>63206</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3233,6 +3243,11 @@
           <t>00:00:46.181</t>
         </is>
       </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>71491</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6992,6 +7007,11 @@
           <t>00:02:06.440</t>
         </is>
       </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>42148</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8731,6 +8751,11 @@
           <t>00:04:30.594</t>
         </is>
       </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>71491</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -9181,6 +9206,11 @@
           <t>00:04:21.428</t>
         </is>
       </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>63206</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -10346,6 +10376,11 @@
           <t>00:04:02.900</t>
         </is>
       </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>36159</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -11641,6 +11676,11 @@
           <t>00:01:53.915</t>
         </is>
       </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>42148</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -13321,6 +13361,11 @@
           <t>00:04:12.680</t>
         </is>
       </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>63206</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -13511,6 +13556,11 @@
           <t>00:03:58.091</t>
         </is>
       </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>36159</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -15444,6 +15494,11 @@
           <t>00:03:57.620</t>
         </is>
       </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>79493</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -16668,6 +16723,11 @@
           <t>00:04:15.897</t>
         </is>
       </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>63206</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -18973,6 +19033,11 @@
           <t>00:00:43.249</t>
         </is>
       </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>63206</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -20817,6 +20882,11 @@
           <t>00:00:42.731</t>
         </is>
       </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t>36164</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -22162,6 +22232,11 @@
           <t>00:01:38.621</t>
         </is>
       </c>
+      <c r="R335" t="inlineStr">
+        <is>
+          <t>88676</t>
+        </is>
+      </c>
       <c r="S335" t="inlineStr">
         <is>
           <t>97361</t>
@@ -22574,6 +22649,11 @@
           <t>00:01:59.086</t>
         </is>
       </c>
+      <c r="R341" t="inlineStr">
+        <is>
+          <t>42148</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -23703,6 +23783,11 @@
           <t>00:04:15.338</t>
         </is>
       </c>
+      <c r="R358" t="inlineStr">
+        <is>
+          <t>36159</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -28217,6 +28302,11 @@
       <c r="L428" t="n">
         <v>7</v>
       </c>
+      <c r="R428" t="inlineStr">
+        <is>
+          <t>36164</t>
+        </is>
+      </c>
       <c r="X428" t="inlineStr">
         <is>
           <t>DNS</t>
@@ -30610,6 +30700,11 @@
           <t>00:04:00.167</t>
         </is>
       </c>
+      <c r="R465" t="inlineStr">
+        <is>
+          <t>79493</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -31633,6 +31728,11 @@
           <t>00:04:24.754</t>
         </is>
       </c>
+      <c r="R481" t="inlineStr">
+        <is>
+          <t>63206</t>
+        </is>
+      </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -34745,6 +34845,11 @@
           <t>00:01:47.456</t>
         </is>
       </c>
+      <c r="R528" t="inlineStr">
+        <is>
+          <t>97236</t>
+        </is>
+      </c>
       <c r="S528" t="inlineStr">
         <is>
           <t>74400</t>
@@ -34961,6 +35066,11 @@
           <t>60136</t>
         </is>
       </c>
+      <c r="S531" t="inlineStr">
+        <is>
+          <t>69203</t>
+        </is>
+      </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -36319,6 +36429,11 @@
           <t>00:04:20.148</t>
         </is>
       </c>
+      <c r="R551" t="inlineStr">
+        <is>
+          <t>49832</t>
+        </is>
+      </c>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
@@ -36649,6 +36764,11 @@
           <t>00:04:03.063</t>
         </is>
       </c>
+      <c r="R556" t="inlineStr">
+        <is>
+          <t>79493</t>
+        </is>
+      </c>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
@@ -38351,6 +38471,11 @@
       <c r="L582" t="n">
         <v>8</v>
       </c>
+      <c r="R582" t="inlineStr">
+        <is>
+          <t>42148</t>
+        </is>
+      </c>
       <c r="X582" t="inlineStr">
         <is>
           <t>DNS</t>
@@ -39185,6 +39310,11 @@
           <t>00:01:57.506</t>
         </is>
       </c>
+      <c r="R595" t="inlineStr">
+        <is>
+          <t>53464</t>
+        </is>
+      </c>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
@@ -39558,6 +39688,11 @@
           <t>00:01:54.424</t>
         </is>
       </c>
+      <c r="R601" t="inlineStr">
+        <is>
+          <t>79493</t>
+        </is>
+      </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
@@ -40191,6 +40326,11 @@
           <t>00:01:59.309</t>
         </is>
       </c>
+      <c r="R611" t="inlineStr">
+        <is>
+          <t>53464</t>
+        </is>
+      </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -41596,6 +41736,11 @@
           <t>00:01:52.377</t>
         </is>
       </c>
+      <c r="R632" t="inlineStr">
+        <is>
+          <t>79493</t>
+        </is>
+      </c>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
@@ -41926,6 +42071,11 @@
           <t>00:01:56.430</t>
         </is>
       </c>
+      <c r="R637" t="inlineStr">
+        <is>
+          <t>53464</t>
+        </is>
+      </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
@@ -42785,6 +42935,11 @@
           <t>00:03:27.189</t>
         </is>
       </c>
+      <c r="R650" t="inlineStr">
+        <is>
+          <t>88676</t>
+        </is>
+      </c>
       <c r="S650" t="inlineStr">
         <is>
           <t>97361</t>
@@ -42990,6 +43145,11 @@
           <t>80648</t>
         </is>
       </c>
+      <c r="S653" t="inlineStr">
+        <is>
+          <t>71491</t>
+        </is>
+      </c>
       <c r="X653" t="inlineStr">
         <is>
           <t>DNS</t>
@@ -43267,6 +43427,11 @@
           <t>00:03:46.695</t>
         </is>
       </c>
+      <c r="R657" t="inlineStr">
+        <is>
+          <t>97236</t>
+        </is>
+      </c>
       <c r="S657" t="inlineStr">
         <is>
           <t>74400</t>
@@ -43334,6 +43499,11 @@
           <t>00:03:56.939</t>
         </is>
       </c>
+      <c r="R658" t="inlineStr">
+        <is>
+          <t>69203</t>
+        </is>
+      </c>
       <c r="S658" t="inlineStr">
         <is>
           <t>60136</t>
@@ -44336,6 +44506,11 @@
           <t>42117</t>
         </is>
       </c>
+      <c r="S672" t="inlineStr">
+        <is>
+          <t>53464</t>
+        </is>
+      </c>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr">
@@ -46265,6 +46440,11 @@
       </c>
       <c r="L701" t="n">
         <v>5</v>
+      </c>
+      <c r="R701" t="inlineStr">
+        <is>
+          <t>49832</t>
+        </is>
       </c>
       <c r="X701" t="inlineStr">
         <is>
@@ -46344,7 +46524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D167"/>
+  <dimension ref="A1:D178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50021,6 +50201,248 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>36159</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Ilia</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>SHTOKALOV</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>36164</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Natalia</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>PODOLSKAIA</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>42148</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Svetlana</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>CHERNIGOVSKAYA</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>49832</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Alena</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>KOSTROMITINA</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>53464</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Dmitrii</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>SHAROV</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>63206</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Joaquim</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>MANHIQUE</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>69203</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>PACHECO</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>71491</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Edgar</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>TUTYAN</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>79493</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Jose Ramon</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>PELIER CORDOVA</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>88676</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Artem</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>KOROVIN</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>97236</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Zakhar</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>PETROV</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>